<commit_message>
Update IG build with correct canonical
</commit_message>
<xml_diff>
--- a/StructureDefinition-demo-patient.xlsx
+++ b/StructureDefinition-demo-patient.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://example.org/fhir/demo-ig/StructureDefinition/demo-patient</t>
+    <t>https://lishathomas19.github.io/fhir-ig-lisha-demo/StructureDefinition/demo-patient</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-18T14:07:37+01:00</t>
+    <t>2025-12-23T14:30:43+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -69,7 +69,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>Lisha Thomas (https://github.com/lishathomas19)</t>
+    <t>Lisha Thomas (https://github.com/lishathomas19/fhir-ig-lisha-demo)</t>
   </si>
   <si>
     <t>Lisha Thomas (lishatej7@gmail.com)</t>

</xml_diff>